<commit_message>
Add dog prefab and associated assets; update UI layout and resource loading
- Created new dog prefab with mesh and texture assets.
- Added dog mesh and texture metadata files.
- Updated MainPanel prefab layout for improved positioning and sizing.
- Enhanced resource loading in ResourceCache to include fallback mechanisms for missing prefabs and sprites.
- Updated building and unit configuration Excel files.
</commit_message>
<xml_diff>
--- a/config/excel/Building.xlsx
+++ b/config/excel/Building.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyZiegler\github\ra2\config\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FB950F-340C-4D43-8E4C-175961CB5D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC330B1E-5554-4FB9-B744-029621CBE924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="30885" windowHeight="16065" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1965" yWindow="4755" windowWidth="34560" windowHeight="16065" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConfBuilding" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="113">
   <si>
     <t>ID</t>
   </si>
@@ -51,16 +51,6 @@
     <t>编号</t>
   </si>
   <si>
-    <t>主基地</t>
-  </si>
-  <si>
-    <t>电厂</t>
-  </si>
-  <si>
-    <t>兵营</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Prefab</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -89,10 +79,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>战车工厂</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Size</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -169,10 +155,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>自动攻击范围内的敌人</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Name</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -196,13 +178,6 @@
   </si>
   <si>
     <t>阵营</t>
-  </si>
-  <si>
-    <t>兵营</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>坦克工厂</t>
   </si>
   <si>
     <t>CampID</t>
@@ -232,28 +207,8 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>2,3</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>CreateUnitIDList</t>
     <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>油田</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>油井</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>碉堡</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>主基地</t>
-    <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
     <t>15,0,15</t>
@@ -292,10 +247,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>油井</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>Images/MainBase</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -320,31 +271,11 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>拥有主基地才能建造其他建筑</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>增加电力</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>ProducePower</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>消耗5点电力，可生产步兵单位</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>消耗10点电力，可生产坦克单位</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>生产10点电力，为基地提供电力支持</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>金钱的来源，持续获得金钱</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
@@ -390,10 +321,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>15,0,25;25,0,15</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>15,0,35</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -410,10 +337,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>110,0,100;100,0,110</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>110,0,90</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -443,6 +366,126 @@
   </si>
   <si>
     <t>血条Y偏移</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>萃取站</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>重型装甲装配厂</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>2</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>3</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>轻型载具工场</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>整备营区</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>基础步兵训练与部署中心，用于征召和整编反重装步兵。配备轻武器库、战术模拟室和快速补给通道，支持步兵单位高效投入战场。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>专用于组装与维护高速轻型装甲车辆的制造设施。采用模块化生产线，可快速批量生产獾式坦克，并提供战场损伤修复服务。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>大型工业化厂房，拥有重型吊装设备与复合装甲压制线，专门用于制造和升级重装坦克。结构坚固，具备一定防御能力，通常部署于战线后方。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>前线指挥枢纽</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>战区核心指挥与部署中心，具备通信中继、单位调度和战场感知能力。所有其他作战建筑必须在其控制范围内建造。被摧毁则丧失作战能力。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>资源回收站</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>通过回收战场残骸、处理废弃装备及协调后勤物流获取作战资金。可升级以提升资源转化效率，是经济运转的核心节点。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>模块化动力阵列</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>提供基地所需能源的分布式发电系统，采用混合能源（柴油、燃料电池或小型燃气轮机）。若电力不足，高级建筑将无法运作或生产速度下降。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>复合防御哨塔</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>多用途自动防御工事，配备360°旋转炮塔，可切换高爆弹（对步兵）或穿甲弹（对轻型载具）模式。对重装坦克效果有限，需配合其他单位协同防御。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>废弃</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>资源回收站</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>前线指挥枢纽</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>模块化动力阵列</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>整备营区</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>重型装甲装配厂</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>轻型载具工场</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>25,0,15</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>15,0,25</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Images/LightVehicleFactory</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>100,0,110</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>110,0,100</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>LightVehicleFactory</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -503,7 +546,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -519,6 +562,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.749992370372631"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -563,7 +612,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -591,9 +640,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -620,6 +666,24 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -888,11 +952,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="2" max="3" width="13.125" customWidth="1"/>
-    <col min="4" max="4" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.75" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.625" customWidth="1"/>
     <col min="6" max="6" width="9.25" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.25" bestFit="1" customWidth="1"/>
@@ -909,7 +973,7 @@
     <col min="19" max="19" width="12" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="17.875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="17.625" customWidth="1"/>
-    <col min="22" max="22" width="33.625" customWidth="1"/>
+    <col min="22" max="22" width="39.625" style="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="15" x14ac:dyDescent="0.25">
@@ -920,132 +984,132 @@
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="S1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="U1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="S1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="T1" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="U1" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="V1" s="5" t="s">
-        <v>33</v>
+      <c r="V1" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="P2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="S2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="T2" s="5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="U2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="V2" s="1" t="s">
-        <v>9</v>
+      <c r="V2" s="13" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:22" ht="120" x14ac:dyDescent="0.25">
@@ -1053,70 +1117,70 @@
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="K3" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="M3" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N3" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="R3" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="U3" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="I3" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="J3" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="K3" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="L3" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="M3" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="N3" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="R3" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="S3" s="3" t="s">
+      <c r="V3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="T3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:22" ht="16.5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:22" ht="66" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>1</v>
       </c>
@@ -1127,10 +1191,10 @@
         <v>0</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="F4" s="6">
         <v>5</v>
@@ -1166,7 +1230,7 @@
         <v>2</v>
       </c>
       <c r="Q4" s="6">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="R4" s="6">
         <v>0</v>
@@ -1176,10 +1240,10 @@
       </c>
       <c r="T4" s="2"/>
       <c r="U4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="V4" s="2" t="s">
-        <v>72</v>
+        <v>92</v>
+      </c>
+      <c r="V4" s="18" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="16.5" x14ac:dyDescent="0.3">
@@ -1192,61 +1256,63 @@
       <c r="C5" s="2">
         <v>0</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F5" s="6">
-        <v>0</v>
-      </c>
-      <c r="G5" s="6">
-        <v>0</v>
-      </c>
-      <c r="H5" s="6">
-        <v>0</v>
-      </c>
-      <c r="I5" s="6">
+      <c r="F5" s="22">
+        <v>0</v>
+      </c>
+      <c r="G5" s="22">
+        <v>0</v>
+      </c>
+      <c r="H5" s="22">
+        <v>0</v>
+      </c>
+      <c r="I5" s="22">
         <v>120</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="22">
         <v>100</v>
       </c>
-      <c r="K5" s="6">
-        <v>0</v>
-      </c>
-      <c r="L5" s="2">
-        <v>0</v>
-      </c>
-      <c r="M5" s="2">
-        <v>0</v>
-      </c>
-      <c r="N5" s="2">
-        <v>0</v>
-      </c>
-      <c r="O5" s="6">
-        <v>0</v>
-      </c>
-      <c r="P5" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="6">
-        <v>0</v>
-      </c>
-      <c r="R5" s="6">
-        <v>0</v>
-      </c>
-      <c r="S5" s="6">
-        <v>0</v>
-      </c>
-      <c r="T5" s="2"/>
-      <c r="U5" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="V5" s="2"/>
-    </row>
-    <row r="6" spans="1:22" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="K5" s="22">
+        <v>0</v>
+      </c>
+      <c r="L5" s="21">
+        <v>0</v>
+      </c>
+      <c r="M5" s="21">
+        <v>0</v>
+      </c>
+      <c r="N5" s="21">
+        <v>0</v>
+      </c>
+      <c r="O5" s="22">
+        <v>0</v>
+      </c>
+      <c r="P5" s="22">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="22">
+        <v>0</v>
+      </c>
+      <c r="R5" s="22">
+        <v>0</v>
+      </c>
+      <c r="S5" s="22">
+        <v>0</v>
+      </c>
+      <c r="T5" s="21"/>
+      <c r="U5" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="V5" s="23" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>3</v>
       </c>
@@ -1257,10 +1323,10 @@
         <v>1</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="F6" s="6">
         <v>5</v>
@@ -1305,14 +1371,14 @@
         <v>0</v>
       </c>
       <c r="T6" s="2"/>
-      <c r="U6" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="V6" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="U6" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="V6" s="18" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" ht="66" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>4</v>
       </c>
@@ -1323,10 +1389,10 @@
         <v>1</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="F7" s="6">
         <v>5</v>
@@ -1372,13 +1438,13 @@
       </c>
       <c r="T7" s="2"/>
       <c r="U7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="V7" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22" ht="16.5" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+      <c r="V7" s="18" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>5</v>
       </c>
@@ -1389,10 +1455,10 @@
         <v>1</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="F8" s="4">
         <v>5</v>
@@ -1436,17 +1502,17 @@
       <c r="S8" s="4">
         <v>5</v>
       </c>
-      <c r="T8" s="10">
-        <v>1</v>
-      </c>
-      <c r="U8" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="V8" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="T8" s="9">
+        <v>1</v>
+      </c>
+      <c r="U8" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="V8" s="18" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>6</v>
       </c>
@@ -1457,10 +1523,10 @@
         <v>1</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>14</v>
+        <v>112</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="F9" s="6">
         <v>5</v>
@@ -1493,28 +1559,28 @@
         <v>20</v>
       </c>
       <c r="P9" s="6">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="Q9" s="6">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="R9" s="6">
         <v>0</v>
       </c>
       <c r="S9" s="6">
-        <v>10</v>
-      </c>
-      <c r="T9" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="U9" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="V9" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22" ht="16.5" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="T9" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="U9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="V9" s="18" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="66" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>7</v>
       </c>
@@ -1522,62 +1588,130 @@
         <v>7</v>
       </c>
       <c r="C10" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="F10" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G10" s="6">
-        <v>1500</v>
+        <v>600</v>
       </c>
       <c r="H10" s="6">
-        <v>-5</v>
+        <v>-20</v>
       </c>
       <c r="I10" s="6">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="J10" s="6">
         <v>100</v>
       </c>
       <c r="K10" s="6">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L10" s="2">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="M10" s="2">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N10" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O10" s="6">
         <v>20</v>
       </c>
       <c r="P10" s="6">
+        <v>6</v>
+      </c>
+      <c r="Q10" s="6">
+        <v>800</v>
+      </c>
+      <c r="R10" s="6">
+        <v>0</v>
+      </c>
+      <c r="S10" s="6">
+        <v>5</v>
+      </c>
+      <c r="T10" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="U10" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="V10" s="18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="66" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2">
+        <v>8</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" s="6">
         <v>3</v>
       </c>
-      <c r="Q10" s="6">
-        <v>300</v>
-      </c>
-      <c r="R10" s="6">
-        <v>0</v>
-      </c>
-      <c r="S10" s="6">
-        <v>0</v>
-      </c>
-      <c r="T10" s="2"/>
-      <c r="U10" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="V10" s="2" t="s">
-        <v>35</v>
+      <c r="G11" s="6">
+        <v>1500</v>
+      </c>
+      <c r="H11" s="6">
+        <v>-5</v>
+      </c>
+      <c r="I11" s="6">
+        <v>80</v>
+      </c>
+      <c r="J11" s="6">
+        <v>100</v>
+      </c>
+      <c r="K11" s="6">
+        <v>4</v>
+      </c>
+      <c r="L11" s="2">
+        <v>15</v>
+      </c>
+      <c r="M11" s="2">
+        <v>5000</v>
+      </c>
+      <c r="N11" s="2">
+        <v>4</v>
+      </c>
+      <c r="O11" s="6">
+        <v>20</v>
+      </c>
+      <c r="P11" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q11" s="6">
+        <v>400</v>
+      </c>
+      <c r="R11" s="6">
+        <v>0</v>
+      </c>
+      <c r="S11" s="6">
+        <v>0</v>
+      </c>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="V11" s="18" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1589,16 +1723,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1EAF20F-3871-496D-B5D3-5055E4F35A32}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="7.125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.875" customWidth="1"/>
-    <col min="4" max="4" width="21.75" customWidth="1"/>
+    <col min="4" max="4" width="28.875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.25">
@@ -1606,30 +1740,30 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>3</v>
@@ -1638,10 +1772,10 @@
         <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>2</v>
@@ -1650,7 +1784,7 @@
         <v>2</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="120" x14ac:dyDescent="0.25">
@@ -1658,336 +1792,388 @@
         <v>4</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A4" s="10">
+        <v>10</v>
+      </c>
+      <c r="B4" s="11">
+        <v>1</v>
+      </c>
+      <c r="C4" s="11">
+        <v>3</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="11">
-        <v>10</v>
-      </c>
-      <c r="B4" s="12">
-        <v>1</v>
-      </c>
-      <c r="C4" s="12">
+      <c r="E4" s="10">
+        <v>1</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="H4" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A5" s="10">
+        <v>11</v>
+      </c>
+      <c r="B5" s="11">
+        <v>1</v>
+      </c>
+      <c r="C5" s="11">
+        <v>4</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="10">
+        <v>1</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="H5" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A6" s="10">
+        <v>12</v>
+      </c>
+      <c r="B6" s="11">
+        <v>1</v>
+      </c>
+      <c r="C6" s="11">
+        <v>5</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" s="10">
+        <v>1</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="H6" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A7" s="10">
+        <v>13</v>
+      </c>
+      <c r="B7" s="11">
+        <v>1</v>
+      </c>
+      <c r="C7" s="11">
+        <v>6</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="E7" s="10">
+        <v>1</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="H7" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A8" s="10">
+        <v>14</v>
+      </c>
+      <c r="B8" s="11">
+        <v>1</v>
+      </c>
+      <c r="C8" s="11">
+        <v>7</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="10">
+        <v>1</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="H8" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="33" x14ac:dyDescent="0.3">
+      <c r="A9" s="10">
+        <v>15</v>
+      </c>
+      <c r="B9" s="11">
+        <v>1</v>
+      </c>
+      <c r="C9" s="11">
+        <v>8</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="10">
+        <v>1</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="H9" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A10" s="10">
+        <v>16</v>
+      </c>
+      <c r="B10" s="11">
+        <v>1</v>
+      </c>
+      <c r="C10" s="11">
+        <v>1</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="10">
+        <v>1</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="H10" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A11" s="14">
+        <v>20</v>
+      </c>
+      <c r="B11" s="15">
+        <v>2</v>
+      </c>
+      <c r="C11" s="15">
         <v>3</v>
       </c>
-      <c r="D4" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E4" s="11">
-        <v>1</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="H4" s="12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="11">
-        <v>11</v>
-      </c>
-      <c r="B5" s="12">
-        <v>1</v>
-      </c>
-      <c r="C5" s="12">
+      <c r="D11" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="14">
+        <v>1</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="H11" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A12" s="14">
+        <v>21</v>
+      </c>
+      <c r="B12" s="15">
+        <v>2</v>
+      </c>
+      <c r="C12" s="15">
         <v>4</v>
       </c>
-      <c r="D5" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="E5" s="11">
-        <v>1</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="G5" s="12" t="s">
+      <c r="D12" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="14">
+        <v>1</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H12" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A13" s="14">
+        <v>22</v>
+      </c>
+      <c r="B13" s="15">
+        <v>2</v>
+      </c>
+      <c r="C13" s="15">
+        <v>5</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" s="14">
+        <v>1</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="H13" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A14" s="14">
+        <v>23</v>
+      </c>
+      <c r="B14" s="15">
+        <v>2</v>
+      </c>
+      <c r="C14" s="15">
         <v>6</v>
       </c>
-      <c r="H5" s="12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="11">
-        <v>12</v>
-      </c>
-      <c r="B6" s="12">
-        <v>1</v>
-      </c>
-      <c r="C6" s="12">
-        <v>5</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="E6" s="11">
-        <v>1</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="H6" s="12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="11">
-        <v>13</v>
-      </c>
-      <c r="B7" s="12">
-        <v>1</v>
-      </c>
-      <c r="C7" s="12">
-        <v>6</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="E7" s="11">
-        <v>1</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" s="12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="33" x14ac:dyDescent="0.3">
-      <c r="A8" s="11">
-        <v>14</v>
-      </c>
-      <c r="B8" s="12">
-        <v>1</v>
-      </c>
-      <c r="C8" s="12">
+      <c r="D14" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="E14" s="14">
+        <v>1</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="H14" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A15" s="14">
+        <v>24</v>
+      </c>
+      <c r="B15" s="15">
+        <v>2</v>
+      </c>
+      <c r="C15" s="15">
         <v>7</v>
       </c>
-      <c r="D8" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="E8" s="11">
-        <v>1</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="H8" s="12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="11">
-        <v>15</v>
-      </c>
-      <c r="B9" s="12">
-        <v>1</v>
-      </c>
-      <c r="C9" s="12">
-        <v>1</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E9" s="11">
-        <v>1</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="H9" s="12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="15">
-        <v>20</v>
-      </c>
-      <c r="B10" s="16">
+      <c r="D15" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="14">
+        <v>1</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="H15" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="33" x14ac:dyDescent="0.3">
+      <c r="A16" s="14">
+        <v>25</v>
+      </c>
+      <c r="B16" s="15">
         <v>2</v>
       </c>
-      <c r="C10" s="16">
-        <v>3</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" s="15">
-        <v>1</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="G10" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="H10" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="15">
-        <v>21</v>
-      </c>
-      <c r="B11" s="16">
+      <c r="C16" s="15">
+        <v>8</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="E16" s="14">
+        <v>1</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="H16" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A17" s="14">
+        <v>26</v>
+      </c>
+      <c r="B17" s="15">
         <v>2</v>
       </c>
-      <c r="C11" s="16">
-        <v>4</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="E11" s="15">
-        <v>1</v>
-      </c>
-      <c r="F11" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="G11" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="H11" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A12" s="15">
-        <v>22</v>
-      </c>
-      <c r="B12" s="16">
-        <v>2</v>
-      </c>
-      <c r="C12" s="16">
-        <v>5</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="E12" s="15">
-        <v>1</v>
-      </c>
-      <c r="F12" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="G12" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="H12" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A13" s="15">
-        <v>23</v>
-      </c>
-      <c r="B13" s="16">
-        <v>2</v>
-      </c>
-      <c r="C13" s="16">
-        <v>6</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="E13" s="15">
-        <v>1</v>
-      </c>
-      <c r="F13" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="G13" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="H13" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="33" x14ac:dyDescent="0.3">
-      <c r="A14" s="15">
-        <v>24</v>
-      </c>
-      <c r="B14" s="16">
-        <v>2</v>
-      </c>
-      <c r="C14" s="16">
-        <v>7</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="E14" s="15">
-        <v>1</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="H14" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A15" s="15">
-        <v>25</v>
-      </c>
-      <c r="B15" s="16">
-        <v>2</v>
-      </c>
-      <c r="C15" s="16">
-        <v>1</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="E15" s="15">
-        <v>1</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="H15" s="16">
+      <c r="C17" s="15">
+        <v>1</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E17" s="14">
+        <v>1</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H17" s="15">
         <v>1</v>
       </c>
     </row>

</xml_diff>